<commit_message>
docs(SCRUM-878): fix Excel sources row heights
</commit_message>
<xml_diff>
--- a/docs/design/reports/character_weapon_mechanics_review_table.xlsx
+++ b/docs/design/reports/character_weapon_mechanics_review_table.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Class Kits" sheetId="1" r:id="R07cc0a435c204e9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapons" sheetId="2" r:id="R740ba73476fc4921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Hotspots" sheetId="3" r:id="R108dcee52048446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rafdfa669be3144c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Class Kits" sheetId="1" r:id="R7109b413caa5473c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapons" sheetId="2" r:id="R5492a9febaab465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Hotspots" sheetId="3" r:id="Rf8f49d2312bd4482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rae892c5af05d4379"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1010,7 +1010,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1714c7f7a0b4058"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6930a34b0e54414"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2114,7 +2114,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a1ffc1d42a240f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1472db76429f4400"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2234,7 +2234,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5576adafcd1e45d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d467911a8a846ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2361,7 +2361,7 @@
         <x:v>Cross-Kit Review Hotspots</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="31.5" customHeight="1">
+    <x:row r="10" ht="87" customHeight="1">
       <x:c r="A10" s="35" t="str">
         <x:v>Source 1</x:v>
       </x:c>
@@ -2375,7 +2375,7 @@
         <x:v>scripts/progression_data_weapons.gd: current WEAPONS_BY_CLASS and weapon configs.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="31.5" customHeight="1">
+    <x:row r="11" ht="87" customHeight="1">
       <x:c r="A11" s="35" t="str">
         <x:v>Source 2</x:v>
       </x:c>
@@ -2389,7 +2389,7 @@
         <x:v>scripts/progression_data_characters.gd: character names, base class identity and weapon identity text.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="31.5" customHeight="1">
+    <x:row r="12" ht="87" customHeight="1">
       <x:c r="A12" s="35" t="str">
         <x:v>Source 3</x:v>
       </x:c>
@@ -2403,7 +2403,7 @@
         <x:v>scripts/class_weapon.gd, scripts/berserk_weapon.gd, scripts/summoner_weapon.gd, scripts/player.gd: runtime attack modes, deploy/summon/drain/block hooks and scaling helpers.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="31.5" customHeight="1">
+    <x:row r="13" ht="87" customHeight="1">
       <x:c r="A13" s="35" t="str">
         <x:v>Source 4</x:v>
       </x:c>
@@ -2417,7 +2417,7 @@
         <x:v>docs/design/systems/characters_weapons.md, docs/design/mechanics_extract.md, docs/design/systems/combat.md: current system documentation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="31.5" customHeight="1">
+    <x:row r="14" ht="87" customHeight="1">
       <x:c r="A14" s="38" t="str">
         <x:v>Source 5</x:v>
       </x:c>
@@ -2438,7 +2438,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f867fcc7b744d4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4c0b1e293e44cf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>